<commit_message>
Added notebooks and numpy practice files
</commit_message>
<xml_diff>
--- a/AI_ML_Daily_Tracker.xlsx
+++ b/AI_ML_Daily_Tracker.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2178" uniqueCount="774">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2189" uniqueCount="774">
   <si>
     <t>🤖  AI / ML ENGINEER – 12-MONTH STREAK TRACKER</t>
   </si>
@@ -4928,27 +4928,27 @@
     <row r="6" ht="49.5" customHeight="1" spans="2:12">
       <c r="B6" s="89">
         <f>'📅 Tracker'!P2</f>
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="C6" s="89"/>
       <c r="D6" s="90">
         <f>'📅 Tracker'!P3</f>
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="E6" s="90"/>
       <c r="F6" s="91">
         <f>'📅 Tracker'!P4</f>
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="G6" s="91"/>
       <c r="H6" s="92">
         <f>'📅 Tracker'!P5</f>
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="I6" s="92"/>
       <c r="J6" s="93">
         <f>'📅 Tracker'!P6</f>
-        <v>14.8809523809524</v>
+        <v>18.1547619047619</v>
       </c>
       <c r="K6" s="93"/>
     </row>
@@ -5005,11 +5005,11 @@
       </c>
       <c r="H10" s="100">
         <f>COUNTIFS('📅 Tracker'!G:G,"Phase 1",'📅 Tracker'!H:H,"✓")</f>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="I10" s="101">
         <f>IFERROR(H10/56,0)</f>
-        <v>0.875</v>
+        <v>0.982142857142857</v>
       </c>
       <c r="J10" s="101"/>
       <c r="K10" s="101"/>
@@ -5031,11 +5031,11 @@
       </c>
       <c r="H11" s="105">
         <f>COUNTIFS('📅 Tracker'!G:G,"Phase 2",'📅 Tracker'!H:H,"✓")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I11" s="106">
         <f>IFERROR(H11/28,0)</f>
-        <v>0.0357142857142857</v>
+        <v>0.214285714285714</v>
       </c>
       <c r="J11" s="106"/>
       <c r="K11" s="106"/>
@@ -5350,7 +5350,7 @@
       </c>
       <c r="P2" s="29">
         <f>COUNTIF(H3:H402,"✓")</f>
-        <v>50</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="2:19">
@@ -5386,7 +5386,7 @@
       </c>
       <c r="P3" s="29">
         <f>336-P2</f>
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="R3" s="37">
         <v>46074</v>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="P4" s="29">
         <f>IFERROR(MATCH(FALSE(),EXACT(H3:H338,"✓"),0)-1,COUNTIF(H3:H338,"✓"))</f>
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="R4" s="37">
         <v>46410</v>
@@ -5470,7 +5470,7 @@
       </c>
       <c r="P5" s="29">
         <f>P2</f>
-        <v>50</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" ht="37.5" customHeight="1" spans="2:19">
@@ -5506,7 +5506,7 @@
       </c>
       <c r="P6" s="38">
         <f>IFERROR(P2/336*100,0)</f>
-        <v>14.8809523809524</v>
+        <v>18.1547619047619</v>
       </c>
     </row>
     <row r="7" ht="37.5" customHeight="1" spans="2:19">
@@ -6569,7 +6569,9 @@
       <c r="G46" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="H46" s="35"/>
+      <c r="H46" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I46" s="36" t="s">
         <v>133</v>
       </c>
@@ -6596,7 +6598,9 @@
       <c r="G47" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="H47" s="35"/>
+      <c r="H47" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I47" s="36" t="s">
         <v>135</v>
       </c>
@@ -6650,7 +6654,9 @@
       <c r="G49" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="H49" s="35"/>
+      <c r="H49" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I49" s="36" t="s">
         <v>139</v>
       </c>
@@ -6833,7 +6839,9 @@
       <c r="G56" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="H56" s="35"/>
+      <c r="H56" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I56" s="36" t="s">
         <v>151</v>
       </c>
@@ -6860,7 +6868,9 @@
       <c r="G57" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="H57" s="35"/>
+      <c r="H57" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I57" s="36" t="s">
         <v>153</v>
       </c>
@@ -7072,7 +7082,9 @@
       <c r="G65" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="H65" s="35"/>
+      <c r="H65" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I65" s="36" t="s">
         <v>167</v>
       </c>
@@ -7163,7 +7175,9 @@
       <c r="G70" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="H70" s="35"/>
+      <c r="H70" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I70" s="36" t="s">
         <v>173</v>
       </c>
@@ -7190,7 +7204,9 @@
       <c r="G71" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="H71" s="35"/>
+      <c r="H71" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I71" s="36" t="s">
         <v>175</v>
       </c>
@@ -7217,7 +7233,9 @@
       <c r="G72" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="H72" s="35"/>
+      <c r="H72" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I72" s="36" t="s">
         <v>177</v>
       </c>
@@ -7244,7 +7262,9 @@
       <c r="G73" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="H73" s="35"/>
+      <c r="H73" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I73" s="36" t="s">
         <v>179</v>
       </c>
@@ -7271,7 +7291,9 @@
       <c r="G74" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="H74" s="35"/>
+      <c r="H74" s="35" t="s">
+        <v>49</v>
+      </c>
       <c r="I74" s="36" t="s">
         <v>181</v>
       </c>

</xml_diff>